<commit_message>
Menambahkan kolom semester dan kelas pada model, controller, dan tampilan jadwal. Memperbarui template impor CSV dan Excel untuk mencakup semester dan kelas. Menambahkan validasi untuk semester dan kelas di controller.
</commit_message>
<xml_diff>
--- a/public/templates/jadwal_import_template.xlsx
+++ b/public/templates/jadwal_import_template.xlsx
@@ -8,8 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Import" sheetId="1" r:id="rId4"/>
-    <sheet name="Laboratorium" sheetId="2" r:id="rId5"/>
-    <sheet name="Program Studi" sheetId="3" r:id="rId6"/>
+    <sheet name="Pilihan" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -17,41 +16,53 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="93">
   <si>
     <t>laboratorium</t>
   </si>
   <si>
+    <t>Laboratorium Komputer ICT Lantai 1</t>
+  </si>
+  <si>
     <t>program_studi</t>
   </si>
   <si>
+    <t>Informatika</t>
+  </si>
+  <si>
     <t>mata_kuliah</t>
   </si>
   <si>
+    <t>Nama Mata Kuliah</t>
+  </si>
+  <si>
+    <t>semester</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>kelas</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
     <t>tanggal</t>
   </si>
   <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
     <t>jam</t>
   </si>
   <si>
+    <t>08:00</t>
+  </si>
+  <si>
     <t>jam_selesai</t>
   </si>
   <si>
-    <t>Laboratorium Komputer ICT Lantai 1</t>
-  </si>
-  <si>
-    <t>Informatika</t>
-  </si>
-  <si>
-    <t>Nama Mata Kuliah</t>
-  </si>
-  <si>
-    <t>2026-09-28</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
     <t>10:50</t>
   </si>
   <si>
@@ -98,6 +109,192 @@
   </si>
   <si>
     <t>Teknologi Pangan</t>
+  </si>
+  <si>
+    <t>3D Design</t>
+  </si>
+  <si>
+    <t>Algorithms and Data Structures</t>
+  </si>
+  <si>
+    <t>AR/VR</t>
+  </si>
+  <si>
+    <t>Asuhan Gizi dan Dietetik PTM Praktikum A</t>
+  </si>
+  <si>
+    <t>Asuhan Gizi dan Dietetik PTM Praktikum B</t>
+  </si>
+  <si>
+    <t>Bakery and Confectionary Technology</t>
+  </si>
+  <si>
+    <t>Basic Chemistry Lab</t>
+  </si>
+  <si>
+    <t>Basic Chemistry Laboratory</t>
+  </si>
+  <si>
+    <t>Big Data for Business</t>
+  </si>
+  <si>
+    <t>Biology Lab</t>
+  </si>
+  <si>
+    <t>Business Intelligence A1</t>
+  </si>
+  <si>
+    <t>Business Intelligence A2</t>
+  </si>
+  <si>
+    <t>Business Statistic II</t>
+  </si>
+  <si>
+    <t>Computer network</t>
+  </si>
+  <si>
+    <t>Data Mining</t>
+  </si>
+  <si>
+    <t>Data Mining &amp; Warehouse</t>
+  </si>
+  <si>
+    <t>Data Processing &amp; Visualization</t>
+  </si>
+  <si>
+    <t>Enterprise Resource Planning (ERP)</t>
+  </si>
+  <si>
+    <t>Ethical Hacking for Business</t>
+  </si>
+  <si>
+    <t>Evaluasi Nilai Gizi Pada Pengolahan</t>
+  </si>
+  <si>
+    <t>Financial Information System</t>
+  </si>
+  <si>
+    <t>Financial Information System (5 DM)</t>
+  </si>
+  <si>
+    <t>Food Preservation</t>
+  </si>
+  <si>
+    <t>Food Sciences Lab</t>
+  </si>
+  <si>
+    <t>Functional Food Development</t>
+  </si>
+  <si>
+    <t>Game Programming</t>
+  </si>
+  <si>
+    <t>GDDK praktikum A</t>
+  </si>
+  <si>
+    <t>GDDK praktikum B</t>
+  </si>
+  <si>
+    <t>Graphic Design</t>
+  </si>
+  <si>
+    <t>Hukum Dagang &amp; Investasi</t>
+  </si>
+  <si>
+    <t>Implementation System and Testing</t>
+  </si>
+  <si>
+    <t>Integrated Business System 1 A</t>
+  </si>
+  <si>
+    <t>International Business Strategy</t>
+  </si>
+  <si>
+    <t>Introduction to Economics</t>
+  </si>
+  <si>
+    <t>Kimia Pangan</t>
+  </si>
+  <si>
+    <t>Kimia Pangan &amp; Pengolahan</t>
+  </si>
+  <si>
+    <t>Leadership for Business A</t>
+  </si>
+  <si>
+    <t>Mikrobiologi Umum</t>
+  </si>
+  <si>
+    <t>Operating system</t>
+  </si>
+  <si>
+    <t>Packaging and Product Design</t>
+  </si>
+  <si>
+    <t>Pemrograman Web Lanjut</t>
+  </si>
+  <si>
+    <t>Penilaian Status Gizi (PSG)</t>
+  </si>
+  <si>
+    <t>PKP praktikum A</t>
+  </si>
+  <si>
+    <t>PKP praktikum B</t>
+  </si>
+  <si>
+    <t>PSG praktikum A</t>
+  </si>
+  <si>
+    <t>PSG praktikum B</t>
+  </si>
+  <si>
+    <t>Satuan Operasi Rekayasa Pangan 1</t>
+  </si>
+  <si>
+    <t>Smart City</t>
+  </si>
+  <si>
+    <t>State Science</t>
+  </si>
+  <si>
+    <t>Statistics</t>
+  </si>
+  <si>
+    <t>Teknologi Minuman dan Bahan Penyegar</t>
+  </si>
+  <si>
+    <t>UI/UX</t>
+  </si>
+  <si>
+    <t>Web Development A1</t>
+  </si>
+  <si>
+    <t>Web Development A2</t>
+  </si>
+  <si>
+    <t>Web Programming 1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
   </si>
 </sst>
 </file>
@@ -151,8 +348,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -453,58 +651,86 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="41.133" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="16.425" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="10.569" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="6.998" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="6.998" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="13.997" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
       </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Pilihan tidak valid" error="Pilih nilai dari daftar." sqref="A2:A300">
+      <formula1>=Pilihan!$A$2:$A$12</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Pilihan tidak valid" error="Pilih nilai dari daftar." sqref="B2:B300">
+      <formula1>=Pilihan!$B$2:$B$7</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Pilihan tidak valid" error="Pilih nilai dari daftar." sqref="C2:C300">
+      <formula1>=Pilihan!$C$2:$C$56</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Pilihan tidak valid" error="Pilih nilai dari daftar." sqref="D2:D300">
+      <formula1>=Pilihan!$D$2:$D$9</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
@@ -525,132 +751,377 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="41.133" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="36.42" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="48.274" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="10.569" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="36.42" bestFit="true" customWidth="true" style="0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>26</v>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="C18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="C19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="C23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="C24" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="C25" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="C26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="C27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="C28" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="C29" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="C31" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="C32" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="C33" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="C34" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="C36" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="C37" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="C38" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="C40" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="C41" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="C42" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="C43" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="C44" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="C45" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="C46" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="C47" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="C48" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="C49" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="C50" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="C51" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="C52" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="C53" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="C54" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="C55" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="C56" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>